<commit_message>
fix(v3): credit Uniswap-V3 fee collections — Grove E12 August was −$49,708, is +$12,139 (#188)
Co-authored-by: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-08/grove_settlement_august_2026.xlsx
+++ b/settlements/grove/2026-08/grove_settlement_august_2026.xlsx
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>4913183.004893322</v>
+        <v>4975029.896919321</v>
       </c>
     </row>
     <row r="5">
@@ -527,7 +527,7 @@
     <row r="8">
       <c r="A8" t="inlineStr"/>
       <c r="B8" s="4" t="n">
-        <v>5020343.444351727</v>
+        <v>5082190.336377727</v>
       </c>
     </row>
     <row r="10">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>4913183.004893322</v>
+        <v>4975029.896919321</v>
       </c>
     </row>
     <row r="22">
@@ -641,7 +641,7 @@
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" s="4" t="n">
-        <v>1192578.160567039</v>
+        <v>1254425.05259304</v>
       </c>
     </row>
     <row r="25">
@@ -676,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-09-02T03:04:03+00:00</t>
+          <t>2026-09-02T13:58:14+00:00</t>
         </is>
       </c>
     </row>
@@ -1011,13 +1011,13 @@
         <v>1</v>
       </c>
       <c r="N4" s="5" t="n">
-        <v>932882.3997984963</v>
+        <v>932905.426134183</v>
       </c>
       <c r="O4" s="5" t="n">
-        <v>932882.3997984963</v>
+        <v>932905.426134183</v>
       </c>
       <c r="P4" s="5" t="n">
-        <v>-458393.5097984963</v>
+        <v>-458416.536134183</v>
       </c>
       <c r="Q4" s="5" t="n">
         <v>0</v>
@@ -1080,13 +1080,13 @@
         <v>1</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>800103.7774898543</v>
+        <v>800123.5264508901</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>800103.7774898543</v>
+        <v>800123.5264508901</v>
       </c>
       <c r="P5" s="5" t="n">
-        <v>342954.5098771617</v>
+        <v>342934.7609161259</v>
       </c>
       <c r="Q5" s="5" t="n">
         <v>0</v>
@@ -1145,13 +1145,13 @@
         <v>1</v>
       </c>
       <c r="N6" s="5" t="n">
-        <v>626964.9135801707</v>
+        <v>626980.3889547378</v>
       </c>
       <c r="O6" s="5" t="n">
-        <v>626964.9135801707</v>
+        <v>626980.3889547378</v>
       </c>
       <c r="P6" s="5" t="n">
-        <v>113207.6931169944</v>
+        <v>113192.2177424274</v>
       </c>
       <c r="Q6" s="5" t="n">
         <v>0</v>
@@ -1210,13 +1210,13 @@
         <v>1</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>399434.2517882582</v>
+        <v>399444.1110236435</v>
       </c>
       <c r="O7" s="5" t="n">
-        <v>399434.2517882582</v>
+        <v>399444.1110236435</v>
       </c>
       <c r="P7" s="5" t="n">
-        <v>171212.5125567601</v>
+        <v>171202.6533213748</v>
       </c>
       <c r="Q7" s="5" t="n">
         <v>0</v>
@@ -1275,13 +1275,13 @@
         <v>1</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>314850.0143653172</v>
+        <v>314857.7858080235</v>
       </c>
       <c r="O8" s="5" t="n">
-        <v>314850.0143653172</v>
+        <v>314857.7858080235</v>
       </c>
       <c r="P8" s="5" t="n">
-        <v>154425.0856346827</v>
+        <v>154417.3141919765</v>
       </c>
       <c r="Q8" s="5" t="n">
         <v>0</v>
@@ -1340,13 +1340,13 @@
         <v>1</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>260598.240872972</v>
+        <v>260604.6732191873</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>260598.240872972</v>
+        <v>260604.6732191873</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v>46359.79987171225</v>
+        <v>46353.36752549692</v>
       </c>
       <c r="Q9" s="5" t="n">
         <v>0</v>
@@ -1405,13 +1405,13 @@
         <v>1</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>84655.87492409915</v>
+        <v>84657.96448500658</v>
       </c>
       <c r="O10" s="5" t="n">
-        <v>84655.87492409915</v>
+        <v>84657.96448500658</v>
       </c>
       <c r="P10" s="5" t="n">
-        <v>138280.3950759009</v>
+        <v>138278.3055149934</v>
       </c>
       <c r="Q10" s="5" t="n">
         <v>0</v>
@@ -1452,31 +1452,31 @@
         <v>3950291.894712</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>-49708.105287</v>
+        <v>12138.786739</v>
       </c>
       <c r="I11" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>-49708.105287</v>
+        <v>12138.786739</v>
       </c>
       <c r="K11" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>26605619.71155881</v>
+        <v>26575693.79606235</v>
       </c>
       <c r="M11" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>81644.45487829178</v>
+        <v>81554.63442129105</v>
       </c>
       <c r="O11" s="5" t="n">
-        <v>81644.45487829178</v>
+        <v>81554.63442129105</v>
       </c>
       <c r="P11" s="5" t="n">
-        <v>-131352.5601652918</v>
+        <v>-69415.84768229105</v>
       </c>
       <c r="Q11" s="5" t="n">
         <v>0</v>
@@ -1535,13 +1535,13 @@
         <v>1</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>74248.27796154158</v>
+        <v>74250.11063173974</v>
       </c>
       <c r="O12" s="5" t="n">
-        <v>74248.27796154158</v>
+        <v>74250.11063173974</v>
       </c>
       <c r="P12" s="5" t="n">
-        <v>-74082.98696419342</v>
+        <v>-74084.81963439159</v>
       </c>
       <c r="Q12" s="5" t="n">
         <v>0</v>
@@ -1600,13 +1600,13 @@
         <v>1</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>74067.55215920263</v>
+        <v>74069.38036854593</v>
       </c>
       <c r="O13" s="5" t="n">
-        <v>74067.55215920263</v>
+        <v>74069.38036854593</v>
       </c>
       <c r="P13" s="5" t="n">
-        <v>59301.90163777841</v>
+        <v>59300.07342843512</v>
       </c>
       <c r="Q13" s="5" t="n">
         <v>0</v>
@@ -1665,13 +1665,13 @@
         <v>1</v>
       </c>
       <c r="N14" s="5" t="n">
-        <v>38358.65118132419</v>
+        <v>38359.59798788714</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>38358.65118132419</v>
+        <v>38359.59798788714</v>
       </c>
       <c r="P14" s="5" t="n">
-        <v>-38358.65118132419</v>
+        <v>-38359.59798788714</v>
       </c>
       <c r="Q14" s="5" t="n">
         <v>0</v>
@@ -1730,13 +1730,13 @@
         <v>1</v>
       </c>
       <c r="N15" s="5" t="n">
-        <v>25740.24381029635</v>
+        <v>25740.8791567181</v>
       </c>
       <c r="O15" s="5" t="n">
-        <v>25740.24381029635</v>
+        <v>25740.8791567181</v>
       </c>
       <c r="P15" s="5" t="n">
-        <v>10793.23697622316</v>
+        <v>10792.6016298014</v>
       </c>
       <c r="Q15" s="5" t="n">
         <v>0</v>
@@ -1795,13 +1795,13 @@
         <v>1</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>6940.272388632459</v>
+        <v>6940.443695371456</v>
       </c>
       <c r="O16" s="5" t="n">
-        <v>6940.272388632459</v>
+        <v>6940.443695371456</v>
       </c>
       <c r="P16" s="5" t="n">
-        <v>382.6521646229415</v>
+        <v>382.4808578839442</v>
       </c>
       <c r="Q16" s="5" t="n">
         <v>0</v>
@@ -1860,13 +1860,13 @@
         <v>1</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>85.01935484926022</v>
+        <v>85.02145338194242</v>
       </c>
       <c r="O17" s="5" t="n">
-        <v>85.01935484926022</v>
+        <v>85.02145338194242</v>
       </c>
       <c r="P17" s="5" t="n">
-        <v>-85.01935484926022</v>
+        <v>-85.02145338194242</v>
       </c>
       <c r="Q17" s="5" t="n">
         <v>0</v>
@@ -1925,13 +1925,13 @@
         <v>1</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>30.89859578446769</v>
+        <v>30.89935845448798</v>
       </c>
       <c r="O18" s="5" t="n">
-        <v>30.89859578446769</v>
+        <v>30.89935845448798</v>
       </c>
       <c r="P18" s="5" t="n">
-        <v>-30.89859578446769</v>
+        <v>-30.89935845448798</v>
       </c>
       <c r="Q18" s="5" t="n">
         <v>0</v>
@@ -1990,13 +1990,13 @@
         <v>1</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>0.001133446220342351</v>
+        <v>0.001133474197194694</v>
       </c>
       <c r="O19" s="5" t="n">
-        <v>0.001133446220342351</v>
+        <v>0.001133474197194694</v>
       </c>
       <c r="P19" s="5" t="n">
-        <v>-0.0002576582571075914</v>
+        <v>-0.0002576862339599341</v>
       </c>
       <c r="Q19" s="5" t="n">
         <v>0</v>
@@ -2055,13 +2055,13 @@
         <v>1</v>
       </c>
       <c r="N20" s="5" t="n">
-        <v>4.374209633258725e-05</v>
+        <v>4.374317601872348e-05</v>
       </c>
       <c r="O20" s="5" t="n">
-        <v>4.374209633258725e-05</v>
+        <v>4.374317601872348e-05</v>
       </c>
       <c r="P20" s="5" t="n">
-        <v>-2.719636373165225e-05</v>
+        <v>-2.719744341778848e-05</v>
       </c>
       <c r="Q20" s="5" t="n">
         <v>0</v>
@@ -2120,13 +2120,13 @@
         <v>1</v>
       </c>
       <c r="N21" s="5" t="n">
-        <v>3.068692094505935e-09</v>
+        <v>3.068767839030971e-09</v>
       </c>
       <c r="O21" s="5" t="n">
-        <v>3.068692094505935e-09</v>
+        <v>3.068767839030971e-09</v>
       </c>
       <c r="P21" s="5" t="n">
-        <v>-3.068692094505935e-09</v>
+        <v>-3.068767839030971e-09</v>
       </c>
       <c r="Q21" s="5" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Grove E41: cost of funds was charged on $12.5M that only arrived on Aug 31 — and show the time-weighted average in summary.md (#189)
Co-authored-by: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-08/grove_settlement_august_2026.xlsx
+++ b/settlements/grove/2026-08/grove_settlement_august_2026.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-09-02T13:58:14+00:00</t>
+          <t>2026-09-02T19:50:48+00:00</t>
         </is>
       </c>
     </row>
@@ -1011,13 +1011,13 @@
         <v>1</v>
       </c>
       <c r="N4" s="5" t="n">
-        <v>932905.426134183</v>
+        <v>939858.3303508102</v>
       </c>
       <c r="O4" s="5" t="n">
-        <v>932905.426134183</v>
+        <v>939858.3303508102</v>
       </c>
       <c r="P4" s="5" t="n">
-        <v>-458416.536134183</v>
+        <v>-465369.4403508102</v>
       </c>
       <c r="Q4" s="5" t="n">
         <v>0</v>
@@ -1080,13 +1080,13 @@
         <v>1</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>800123.5264508901</v>
+        <v>806086.8128516736</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>800123.5264508901</v>
+        <v>806086.8128516736</v>
       </c>
       <c r="P5" s="5" t="n">
-        <v>342934.7609161259</v>
+        <v>336971.4745153424</v>
       </c>
       <c r="Q5" s="5" t="n">
         <v>0</v>
@@ -1145,13 +1145,13 @@
         <v>1</v>
       </c>
       <c r="N6" s="5" t="n">
-        <v>626980.3889547378</v>
+        <v>631653.246961546</v>
       </c>
       <c r="O6" s="5" t="n">
-        <v>626980.3889547378</v>
+        <v>631653.246961546</v>
       </c>
       <c r="P6" s="5" t="n">
-        <v>113192.2177424274</v>
+        <v>108519.3597356191</v>
       </c>
       <c r="Q6" s="5" t="n">
         <v>0</v>
@@ -1210,13 +1210,13 @@
         <v>1</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>399444.1110236435</v>
+        <v>402421.150888608</v>
       </c>
       <c r="O7" s="5" t="n">
-        <v>399444.1110236435</v>
+        <v>402421.150888608</v>
       </c>
       <c r="P7" s="5" t="n">
-        <v>171202.6533213748</v>
+        <v>168225.6134564103</v>
       </c>
       <c r="Q7" s="5" t="n">
         <v>0</v>
@@ -1275,13 +1275,13 @@
         <v>1</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>314857.7858080235</v>
+        <v>317204.4074110879</v>
       </c>
       <c r="O8" s="5" t="n">
-        <v>314857.7858080235</v>
+        <v>317204.4074110879</v>
       </c>
       <c r="P8" s="5" t="n">
-        <v>154417.3141919765</v>
+        <v>152070.692588912</v>
       </c>
       <c r="Q8" s="5" t="n">
         <v>0</v>
@@ -1340,13 +1340,13 @@
         <v>1</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>260604.6732191873</v>
+        <v>262546.9486959277</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>260604.6732191873</v>
+        <v>262546.9486959277</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v>46353.36752549692</v>
+        <v>44411.09204875655</v>
       </c>
       <c r="Q9" s="5" t="n">
         <v>0</v>
@@ -1405,13 +1405,13 @@
         <v>1</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>84657.96448500658</v>
+        <v>85288.91667131556</v>
       </c>
       <c r="O10" s="5" t="n">
-        <v>84657.96448500658</v>
+        <v>85288.91667131556</v>
       </c>
       <c r="P10" s="5" t="n">
-        <v>138278.3055149934</v>
+        <v>137647.3533286844</v>
       </c>
       <c r="Q10" s="5" t="n">
         <v>0</v>
@@ -1470,13 +1470,13 @@
         <v>1</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>81554.63442129105</v>
+        <v>82162.45762144438</v>
       </c>
       <c r="O11" s="5" t="n">
-        <v>81554.63442129105</v>
+        <v>82162.45762144438</v>
       </c>
       <c r="P11" s="5" t="n">
-        <v>-69415.84768229105</v>
+        <v>-70023.67088244438</v>
       </c>
       <c r="Q11" s="5" t="n">
         <v>0</v>
@@ -1535,13 +1535,13 @@
         <v>1</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>74250.11063173974</v>
+        <v>74803.49352869183</v>
       </c>
       <c r="O12" s="5" t="n">
-        <v>74250.11063173974</v>
+        <v>74803.49352869183</v>
       </c>
       <c r="P12" s="5" t="n">
-        <v>-74084.81963439159</v>
+        <v>-74638.20253134368</v>
       </c>
       <c r="Q12" s="5" t="n">
         <v>0</v>
@@ -1600,13 +1600,13 @@
         <v>1</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>74069.38036854593</v>
+        <v>74621.41629058092</v>
       </c>
       <c r="O13" s="5" t="n">
-        <v>74069.38036854593</v>
+        <v>74621.41629058092</v>
       </c>
       <c r="P13" s="5" t="n">
-        <v>59300.07342843512</v>
+        <v>58748.03750640013</v>
       </c>
       <c r="Q13" s="5" t="n">
         <v>0</v>
@@ -1619,12 +1619,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>E41</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>JTRSY Basin escrow — USDS pending subscription (Diamond PAU)</t>
+          <t>Grove x Steakhouse AUSD (Morpho 4626)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1634,44 +1634,44 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>1000000</v>
+        <v>25197943.54576933</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>12500000</v>
+        <v>0.02838475959697621</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>11500000</v>
+        <v>-25197943.51738457</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0</v>
+        <v>36533.48078651951</v>
       </c>
       <c r="I14" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0</v>
+        <v>36533.48078651951</v>
       </c>
       <c r="K14" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>12500000</v>
+        <v>8388017.767041751</v>
       </c>
       <c r="M14" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N14" s="5" t="n">
-        <v>38359.59798788714</v>
+        <v>25932.7248274739</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>38359.59798788714</v>
+        <v>25932.7248274739</v>
       </c>
       <c r="P14" s="5" t="n">
-        <v>-38359.59798788714</v>
+        <v>10600.7559590456</v>
       </c>
       <c r="Q14" s="5" t="n">
         <v>0</v>
@@ -1684,12 +1684,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>E41</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Grove x Steakhouse AUSD (Morpho 4626)</t>
+          <t>JTRSY Basin escrow — USDS pending subscription (Diamond PAU)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1699,44 +1699,44 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>25197943.54576933</v>
+        <v>1000000</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.02838475959697621</v>
+        <v>12500000</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>-25197943.51738457</v>
+        <v>11500000</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>36533.48078651951</v>
+        <v>0</v>
       </c>
       <c r="I15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>36533.48078651951</v>
+        <v>0</v>
       </c>
       <c r="K15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>8388017.767041751</v>
+        <v>3369516.774752</v>
       </c>
       <c r="M15" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N15" s="5" t="n">
-        <v>25740.8791567181</v>
+        <v>10417.33026180964</v>
       </c>
       <c r="O15" s="5" t="n">
-        <v>25740.8791567181</v>
+        <v>10417.33026180964</v>
       </c>
       <c r="P15" s="5" t="n">
-        <v>10792.6016298014</v>
+        <v>-10417.33026180964</v>
       </c>
       <c r="Q15" s="5" t="n">
         <v>0</v>
@@ -1795,13 +1795,13 @@
         <v>1</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>6940.443695371456</v>
+        <v>6992.170525211838</v>
       </c>
       <c r="O16" s="5" t="n">
-        <v>6940.443695371456</v>
+        <v>6992.170525211838</v>
       </c>
       <c r="P16" s="5" t="n">
-        <v>382.4808578839442</v>
+        <v>330.7540280435622</v>
       </c>
       <c r="Q16" s="5" t="n">
         <v>0</v>
@@ -1814,17 +1814,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>E15</t>
+          <t>E27</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>USDC raw (ALM idle)</t>
+          <t>USDC raw on Base (ALM idle)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>base</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1836,37 +1836,37 @@
         <v>0</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>999.178498</v>
+        <v>0</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>999.178498</v>
+        <v>0</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>-1.4e-23</v>
+        <v>0</v>
       </c>
       <c r="I17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>-1.4e-23</v>
+        <v>0</v>
       </c>
       <c r="K17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L17" s="5" t="n">
-        <v>27705.40420183423</v>
+        <v>161290.3225806452</v>
       </c>
       <c r="M17" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>85.02145338194242</v>
+        <v>498.6514894201883</v>
       </c>
       <c r="O17" s="5" t="n">
-        <v>85.02145338194242</v>
+        <v>498.6514894201883</v>
       </c>
       <c r="P17" s="5" t="n">
-        <v>-85.02145338194242</v>
+        <v>-498.6514894201883</v>
       </c>
       <c r="Q17" s="5" t="n">
         <v>0</v>
@@ -1879,12 +1879,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>E31</t>
+          <t>E15</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>AUSD raw (alt holder idle)</t>
+          <t>USDC raw (ALM idle)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1898,40 +1898,40 @@
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>10068.978846</v>
+        <v>0</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>10068.978846</v>
+        <v>999.178498</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>0</v>
+        <v>999.178498</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0</v>
+        <v>-1.4e-23</v>
       </c>
       <c r="I18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0</v>
+        <v>-1.4e-23</v>
       </c>
       <c r="K18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L18" s="5" t="n">
-        <v>10068.978846</v>
+        <v>27705.40420183423</v>
       </c>
       <c r="M18" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>30.89935845448798</v>
+        <v>85.65511463544451</v>
       </c>
       <c r="O18" s="5" t="n">
-        <v>30.89935845448798</v>
+        <v>85.65511463544451</v>
       </c>
       <c r="P18" s="5" t="n">
-        <v>-30.89935845448798</v>
+        <v>-85.65511463544451</v>
       </c>
       <c r="Q18" s="5" t="n">
         <v>0</v>
@@ -1944,12 +1944,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>E31</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Aave Ethereum RLUSD (aToken)</t>
+          <t>AUSD raw (alt holder idle)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1959,44 +1959,44 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E19" s="5" t="n">
-        <v>0.369358080066628</v>
+        <v>10068.978846</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.3702338680298627</v>
+        <v>10068.978846</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>0.00087578796323476</v>
+        <v>0</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>0.00087578796323476</v>
+        <v>0</v>
       </c>
       <c r="I19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>0.00087578796323476</v>
+        <v>0</v>
       </c>
       <c r="K19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>0.369358080066628</v>
+        <v>10068.978846</v>
       </c>
       <c r="M19" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>0.001133474197194694</v>
+        <v>31.12965005068927</v>
       </c>
       <c r="O19" s="5" t="n">
-        <v>0.001133474197194694</v>
+        <v>31.12965005068927</v>
       </c>
       <c r="P19" s="5" t="n">
-        <v>-0.0002576862339599341</v>
+        <v>-31.12965005068927</v>
       </c>
       <c r="Q19" s="5" t="n">
         <v>0</v>
@@ -2009,12 +2009,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Aave Horizon RWA RLUSD (aToken)</t>
+          <t>Aave Ethereum RLUSD (aToken)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2028,40 +2028,40 @@
         </is>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.01425431258186553</v>
+        <v>0.369358080066628</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>0.01427085831446647</v>
+        <v>0.3702338680298627</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>1.6545732600935e-05</v>
+        <v>0.00087578796323476</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>1.6545732600935e-05</v>
+        <v>0.00087578796323476</v>
       </c>
       <c r="I20" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>1.6545732600935e-05</v>
+        <v>0.00087578796323476</v>
       </c>
       <c r="K20" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L20" s="5" t="n">
-        <v>0.01425431258186553</v>
+        <v>0.369358080066628</v>
       </c>
       <c r="M20" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N20" s="5" t="n">
-        <v>4.374317601872348e-05</v>
+        <v>0.001141921931878552</v>
       </c>
       <c r="O20" s="5" t="n">
-        <v>4.374317601872348e-05</v>
+        <v>0.001141921931878552</v>
       </c>
       <c r="P20" s="5" t="n">
-        <v>-2.719744341778848e-05</v>
+        <v>-0.0002661339686437922</v>
       </c>
       <c r="Q20" s="5" t="n">
         <v>0</v>
@@ -2074,12 +2074,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Aave Horizon RWA USDC (aToken)</t>
+          <t>Aave Horizon RWA RLUSD (aToken)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2093,40 +2093,40 @@
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>1e-06</v>
+        <v>0.01425431258186553</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>1e-06</v>
+        <v>0.01427085831446647</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>0</v>
+        <v>1.6545732600935e-05</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>0</v>
+        <v>1.6545732600935e-05</v>
       </c>
       <c r="I21" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>0</v>
+        <v>1.6545732600935e-05</v>
       </c>
       <c r="K21" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L21" s="5" t="n">
-        <v>1e-06</v>
+        <v>0.01425431258186553</v>
       </c>
       <c r="M21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N21" s="5" t="n">
-        <v>3.068767839030971e-09</v>
+        <v>4.406919203757071e-05</v>
       </c>
       <c r="O21" s="5" t="n">
-        <v>3.068767839030971e-09</v>
+        <v>4.406919203757071e-05</v>
       </c>
       <c r="P21" s="5" t="n">
-        <v>-3.068767839030971e-09</v>
+        <v>-2.752345943663571e-05</v>
       </c>
       <c r="Q21" s="5" t="n">
         <v>0</v>
@@ -2139,12 +2139,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>E5</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Grove x Steakhouse USDC High Yield (Morpho 4626)</t>
+          <t>Aave Horizon RWA USDC (aToken)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2154,14 +2154,14 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
       <c r="G22" s="5" t="n">
         <v>0</v>
@@ -2179,19 +2179,19 @@
         <v>0</v>
       </c>
       <c r="L22" s="5" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
       <c r="M22" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N22" s="5" t="n">
-        <v>0</v>
+        <v>3.091639234405168e-09</v>
       </c>
       <c r="O22" s="5" t="n">
-        <v>0</v>
+        <v>3.091639234405168e-09</v>
       </c>
       <c r="P22" s="5" t="n">
-        <v>0</v>
+        <v>-3.091639234405168e-09</v>
       </c>
       <c r="Q22" s="5" t="n">
         <v>0</v>
@@ -2204,12 +2204,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>E37</t>
+          <t>E5</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Maple syrupUSDC (ERC-4626)</t>
+          <t>Grove x Steakhouse USDC High Yield (Morpho 4626)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2269,12 +2269,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>E30</t>
+          <t>E37</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Uniswap V3 AUSD/USDC pool (NFT positions — alt holder)</t>
+          <t>Maple syrupUSDC (ERC-4626)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E24" s="5" t="n">
@@ -2334,12 +2334,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>E13</t>
+          <t>E30</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>RLUSD raw (ALM idle)</t>
+          <t>Uniswap V3 AUSD/USDC pool (NFT positions — alt holder)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E25" s="5" t="n">
@@ -2399,12 +2399,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>E32</t>
+          <t>E13</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>USDC raw (alt holder idle)</t>
+          <t>RLUSD raw (ALM idle)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2464,12 +2464,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>E16</t>
+          <t>E32</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DAI raw (ALM idle)</t>
+          <t>USDC raw (alt holder idle)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2529,12 +2529,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>E17</t>
+          <t>E16</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>USDS raw / POL (ALM idle — already netted out of utilized)</t>
+          <t>DAI raw (ALM idle)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2572,7 +2572,7 @@
         <v>0</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N28" s="5" t="n">
         <v>0</v>
@@ -2589,21 +2589,17 @@
       <c r="R28" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>CoF excluded (already deducted from utilized)</t>
-        </is>
-      </c>
+      <c r="S28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>E18</t>
+          <t>E17</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>sUSDS raw / POL (ALM idle — Cat B 4626)</t>
+          <t>USDS raw / POL (ALM idle — already netted out of utilized)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2613,7 +2609,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E29" s="5" t="n">
@@ -2641,7 +2637,7 @@
         <v>0</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N29" s="5" t="n">
         <v>0</v>
@@ -2658,17 +2654,21 @@
       <c r="R29" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="S29" t="inlineStr"/>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>CoF excluded (already deducted from utilized)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>E24</t>
+          <t>E18</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Steakhouse High Yield PYUSD (Morpho 4626)</t>
+          <t>sUSDS raw / POL (ALM idle — Cat B 4626)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2728,12 +2728,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>E26</t>
+          <t>E24</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PYUSD raw (ALM idle)</t>
+          <t>Steakhouse High Yield PYUSD (Morpho 4626)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E31" s="5" t="n">
@@ -2793,17 +2793,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>E27</t>
+          <t>E26</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>USDC raw on Base (ALM idle)</t>
+          <t>PYUSD raw (ALM idle)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">

</xml_diff>

<commit_message>
Grove: price ACRDX redemptions at what they settle for, and stop assuming GACLO-1 was flat all month (#191)
Co-authored-by: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-08/grove_settlement_august_2026.xlsx
+++ b/settlements/grove/2026-08/grove_settlement_august_2026.xlsx
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>4975029.896919321</v>
+        <v>4955508.14483875</v>
       </c>
     </row>
     <row r="5">
@@ -527,7 +527,7 @@
     <row r="8">
       <c r="A8" t="inlineStr"/>
       <c r="B8" s="4" t="n">
-        <v>5082190.336377727</v>
+        <v>5062668.584297156</v>
       </c>
     </row>
     <row r="10">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>4975029.896919321</v>
+        <v>4955508.14483875</v>
       </c>
     </row>
     <row r="22">
@@ -641,7 +641,7 @@
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" s="4" t="n">
-        <v>1254425.05259304</v>
+        <v>1234903.300512468</v>
       </c>
     </row>
     <row r="25">
@@ -676,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-09-02T19:50:48+00:00</t>
+          <t>2026-09-02T21:08:28+00:00</t>
         </is>
       </c>
     </row>
@@ -1011,13 +1011,13 @@
         <v>1</v>
       </c>
       <c r="N4" s="5" t="n">
-        <v>939858.3303508102</v>
+        <v>943028.1360796315</v>
       </c>
       <c r="O4" s="5" t="n">
-        <v>939858.3303508102</v>
+        <v>943028.1360796315</v>
       </c>
       <c r="P4" s="5" t="n">
-        <v>-465369.4403508102</v>
+        <v>-468539.2460796316</v>
       </c>
       <c r="Q4" s="5" t="n">
         <v>0</v>
@@ -1080,13 +1080,13 @@
         <v>1</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>806086.8128516736</v>
+        <v>808805.4551350811</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>806086.8128516736</v>
+        <v>808805.4551350811</v>
       </c>
       <c r="P5" s="5" t="n">
-        <v>336971.4745153424</v>
+        <v>334252.8322319349</v>
       </c>
       <c r="Q5" s="5" t="n">
         <v>0</v>
@@ -1145,13 +1145,13 @@
         <v>1</v>
       </c>
       <c r="N6" s="5" t="n">
-        <v>631653.246961546</v>
+        <v>633783.5872651745</v>
       </c>
       <c r="O6" s="5" t="n">
-        <v>631653.246961546</v>
+        <v>633783.5872651745</v>
       </c>
       <c r="P6" s="5" t="n">
-        <v>108519.3597356191</v>
+        <v>106389.0194319907</v>
       </c>
       <c r="Q6" s="5" t="n">
         <v>0</v>
@@ -1210,13 +1210,13 @@
         <v>1</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>402421.150888608</v>
+        <v>403778.3733851193</v>
       </c>
       <c r="O7" s="5" t="n">
-        <v>402421.150888608</v>
+        <v>403778.3733851193</v>
       </c>
       <c r="P7" s="5" t="n">
-        <v>168225.6134564103</v>
+        <v>166868.3909598991</v>
       </c>
       <c r="Q7" s="5" t="n">
         <v>0</v>
@@ -1275,13 +1275,13 @@
         <v>1</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>317204.4074110879</v>
+        <v>318274.2243349256</v>
       </c>
       <c r="O8" s="5" t="n">
-        <v>317204.4074110879</v>
+        <v>318274.2243349256</v>
       </c>
       <c r="P8" s="5" t="n">
-        <v>152070.692588912</v>
+        <v>151000.8756650744</v>
       </c>
       <c r="Q8" s="5" t="n">
         <v>0</v>
@@ -1340,13 +1340,13 @@
         <v>1</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>262546.9486959277</v>
+        <v>263432.4255759914</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>262546.9486959277</v>
+        <v>263432.4255759914</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v>44411.09204875655</v>
+        <v>43525.61516869286</v>
       </c>
       <c r="Q9" s="5" t="n">
         <v>0</v>
@@ -1359,59 +1359,59 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>E21</t>
+          <t>E12</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Galaxy Arch CLO Token (GACLO-1)</t>
+          <t>Uniswap V3 AUSD/USDC pool (NFT positions)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>avalanche_c</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>27586956.37</v>
+        <v>25057232.614785</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>17907834.79</v>
+        <v>29007524.509497</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>-9679121.58</v>
+        <v>3950291.894712</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>222936.27</v>
+        <v>12138.786739</v>
       </c>
       <c r="I10" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>222936.27</v>
+        <v>12138.786739</v>
       </c>
       <c r="K10" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L10" s="5" t="n">
-        <v>27586956.37</v>
+        <v>26575693.79606235</v>
       </c>
       <c r="M10" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>85288.91667131556</v>
+        <v>82439.56218119785</v>
       </c>
       <c r="O10" s="5" t="n">
-        <v>85288.91667131556</v>
+        <v>82439.56218119785</v>
       </c>
       <c r="P10" s="5" t="n">
-        <v>137647.3533286844</v>
+        <v>-70300.77544219786</v>
       </c>
       <c r="Q10" s="5" t="n">
         <v>0</v>
@@ -1424,12 +1424,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>E12</t>
+          <t>E11</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Uniswap V3 AUSD/USDC pool (NFT positions)</t>
+          <t>Curve AUSD/USDC stableswap LP</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1443,40 +1443,40 @@
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>25057232.614785</v>
+        <v>25001934.08299074</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>29007524.509497</v>
+        <v>0</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>3950291.894712</v>
+        <v>-25001934.08299074</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>12138.786739</v>
+        <v>165.2909973481477</v>
       </c>
       <c r="I11" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>12138.786739</v>
+        <v>165.2909973481477</v>
       </c>
       <c r="K11" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>26575693.79606235</v>
+        <v>24195414.74834597</v>
       </c>
       <c r="M11" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>82162.45762144438</v>
+        <v>75055.77893667943</v>
       </c>
       <c r="O11" s="5" t="n">
-        <v>82162.45762144438</v>
+        <v>75055.77893667943</v>
       </c>
       <c r="P11" s="5" t="n">
-        <v>-70023.67088244438</v>
+        <v>-74890.48793933127</v>
       </c>
       <c r="Q11" s="5" t="n">
         <v>0</v>
@@ -1489,59 +1489,59 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>E11</t>
+          <t>E22</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Curve AUSD/USDC stableswap LP</t>
+          <t>Anemoy Tokenized Apollo Diversified Credit Fund (ACRDX)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>plume</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>25001934.08299074</v>
+        <v>32853651.7342501</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0</v>
+        <v>20703791.96596751</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>-25001934.08299074</v>
+        <v>-12149859.76828259</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>165.2909973481477</v>
+        <v>113847.7017164101</v>
       </c>
       <c r="I12" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>165.2909973481477</v>
+        <v>113847.7017164101</v>
       </c>
       <c r="K12" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>24195414.74834597</v>
+        <v>24150375.46521855</v>
       </c>
       <c r="M12" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>74803.49352869183</v>
+        <v>74916.06409760608</v>
       </c>
       <c r="O12" s="5" t="n">
-        <v>74803.49352869183</v>
+        <v>74916.06409760608</v>
       </c>
       <c r="P12" s="5" t="n">
-        <v>-74638.20253134368</v>
+        <v>38931.63761880402</v>
       </c>
       <c r="Q12" s="5" t="n">
         <v>0</v>
@@ -1554,17 +1554,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>E22</t>
+          <t>E21</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Anemoy Tokenized Apollo Diversified Credit Fund (ACRDX)</t>
+          <t>Galaxy Arch CLO Token (GACLO-1)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>plume</t>
+          <t>avalanche_c</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1573,40 +1573,40 @@
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>32853651.7342501</v>
+        <v>27586956.37</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>20703791.96596751</v>
+        <v>17907834.79</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>-12149859.76828259</v>
+        <v>-9679121.58</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>133369.453796981</v>
+        <v>222936.27</v>
       </c>
       <c r="I13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>133369.453796981</v>
+        <v>222936.27</v>
       </c>
       <c r="K13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>24136521.31858072</v>
+        <v>23527969.90096774</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>74621.41629058092</v>
+        <v>72985.32081730908</v>
       </c>
       <c r="O13" s="5" t="n">
-        <v>74621.41629058092</v>
+        <v>72985.32081730908</v>
       </c>
       <c r="P13" s="5" t="n">
-        <v>58748.03750640013</v>
+        <v>149950.9491826909</v>
       </c>
       <c r="Q13" s="5" t="n">
         <v>0</v>
@@ -1665,13 +1665,13 @@
         <v>1</v>
       </c>
       <c r="N14" s="5" t="n">
-        <v>25932.7248274739</v>
+        <v>26020.18662577641</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>25932.7248274739</v>
+        <v>26020.18662577641</v>
       </c>
       <c r="P14" s="5" t="n">
-        <v>10600.7559590456</v>
+        <v>10513.2941607431</v>
       </c>
       <c r="Q14" s="5" t="n">
         <v>0</v>
@@ -1730,13 +1730,13 @@
         <v>1</v>
       </c>
       <c r="N15" s="5" t="n">
-        <v>10417.33026180964</v>
+        <v>10452.46418793081</v>
       </c>
       <c r="O15" s="5" t="n">
-        <v>10417.33026180964</v>
+        <v>10452.46418793081</v>
       </c>
       <c r="P15" s="5" t="n">
-        <v>-10417.33026180964</v>
+        <v>-10452.46418793081</v>
       </c>
       <c r="Q15" s="5" t="n">
         <v>0</v>
@@ -1795,13 +1795,13 @@
         <v>1</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>6992.170525211838</v>
+        <v>7015.752613567047</v>
       </c>
       <c r="O16" s="5" t="n">
-        <v>6992.170525211838</v>
+        <v>7015.752613567047</v>
       </c>
       <c r="P16" s="5" t="n">
-        <v>330.7540280435622</v>
+        <v>307.1719396883531</v>
       </c>
       <c r="Q16" s="5" t="n">
         <v>0</v>
@@ -1860,13 +1860,13 @@
         <v>1</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>498.6514894201883</v>
+        <v>500.3332624032074</v>
       </c>
       <c r="O17" s="5" t="n">
-        <v>498.6514894201883</v>
+        <v>500.3332624032074</v>
       </c>
       <c r="P17" s="5" t="n">
-        <v>-498.6514894201883</v>
+        <v>-500.3332624032074</v>
       </c>
       <c r="Q17" s="5" t="n">
         <v>0</v>
@@ -1925,13 +1925,13 @@
         <v>1</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>85.65511463544451</v>
+        <v>85.94399867712016</v>
       </c>
       <c r="O18" s="5" t="n">
-        <v>85.65511463544451</v>
+        <v>85.94399867712016</v>
       </c>
       <c r="P18" s="5" t="n">
-        <v>-85.65511463544451</v>
+        <v>-85.94399867712016</v>
       </c>
       <c r="Q18" s="5" t="n">
         <v>0</v>
@@ -1990,13 +1990,13 @@
         <v>1</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>31.12965005068927</v>
+        <v>31.23463921754599</v>
       </c>
       <c r="O19" s="5" t="n">
-        <v>31.12965005068927</v>
+        <v>31.23463921754599</v>
       </c>
       <c r="P19" s="5" t="n">
-        <v>-31.12965005068927</v>
+        <v>-31.23463921754599</v>
       </c>
       <c r="Q19" s="5" t="n">
         <v>0</v>
@@ -2055,13 +2055,13 @@
         <v>1</v>
       </c>
       <c r="N20" s="5" t="n">
-        <v>0.001141921931878552</v>
+        <v>0.001145773225807271</v>
       </c>
       <c r="O20" s="5" t="n">
-        <v>0.001141921931878552</v>
+        <v>0.001145773225807271</v>
       </c>
       <c r="P20" s="5" t="n">
-        <v>-0.0002661339686437922</v>
+        <v>-0.0002699852625725105</v>
       </c>
       <c r="Q20" s="5" t="n">
         <v>0</v>
@@ -2120,13 +2120,13 @@
         <v>1</v>
       </c>
       <c r="N21" s="5" t="n">
-        <v>4.406919203757071e-05</v>
+        <v>4.421782164787919e-05</v>
       </c>
       <c r="O21" s="5" t="n">
-        <v>4.406919203757071e-05</v>
+        <v>4.421782164787919e-05</v>
       </c>
       <c r="P21" s="5" t="n">
-        <v>-2.752345943663571e-05</v>
+        <v>-2.767208904694419e-05</v>
       </c>
       <c r="Q21" s="5" t="n">
         <v>0</v>
@@ -2185,13 +2185,13 @@
         <v>1</v>
       </c>
       <c r="N22" s="5" t="n">
-        <v>3.091639234405168e-09</v>
+        <v>3.102066226899886e-09</v>
       </c>
       <c r="O22" s="5" t="n">
-        <v>3.091639234405168e-09</v>
+        <v>3.102066226899886e-09</v>
       </c>
       <c r="P22" s="5" t="n">
-        <v>-3.091639234405168e-09</v>
+        <v>-3.102066226899886e-09</v>
       </c>
       <c r="Q22" s="5" t="n">
         <v>0</v>

</xml_diff>